<commit_message>
update chungtu data august 2026
</commit_message>
<xml_diff>
--- a/ui/public/sample/sample-chungtu.xlsx
+++ b/ui/public/sample/sample-chungtu.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\vlute\kiemketaisan\ui\public\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B24F0D9E-409B-4C35-A11F-1A0773CF3C7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA7F0E72-6DC5-4DDF-8D5B-3451DB954E24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D2D41EFE-3439-4D12-A44F-8ABA1BF3FB1E}"/>
   </bookViews>
@@ -41,6 +41,30 @@
     <author>hieulth</author>
   </authors>
   <commentList>
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{42F67CE1-8E8A-4B5E-A6B3-DAC7FDA3F5AF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>hieulth:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Không cần phải điền</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="G1" authorId="0" shapeId="0" xr:uid="{83B2D79C-EE88-44EA-9E7D-F1142750BEA8}">
       <text>
         <r>
@@ -126,10 +150,10 @@
     <t>Một trăm hai mươi ba đồng</t>
   </si>
   <si>
-    <t>Đã thanh toán</t>
-  </si>
-  <si>
     <t>Nhà cung cấp</t>
+  </si>
+  <si>
+    <t>Đã nhận</t>
   </si>
 </sst>
 </file>
@@ -557,7 +581,7 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
@@ -570,9 +594,7 @@
       <c r="C2">
         <v>123</v>
       </c>
-      <c r="D2" s="3">
-        <v>46196</v>
-      </c>
+      <c r="D2" s="3"/>
       <c r="E2" t="s">
         <v>8</v>
       </c>
@@ -580,7 +602,7 @@
         <v>9</v>
       </c>
       <c r="G2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -592,7 +614,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{BF5FC730-576E-47FC-B197-EB02620F0831}">
-      <formula1>"Đã thanh toán, Thanh toán một phần, Đã thanh toán nhưng chưa scan, Chưa xác định"</formula1>
+      <formula1>"Đã nhận,Đã duyệt thanh toán,Đã thanh toán"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>